<commit_message>
Automate script for CAAS
</commit_message>
<xml_diff>
--- a/Lab 02/RunningTimeRecording.xlsx
+++ b/Lab 02/RunningTimeRecording.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\MONASH\Year_3_sem_1\FIT3143\Week 04\FIT3143_lab01\Lab 02\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chtay\Documents\FIT3143\FIT3143_lab01\Lab 02\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B57F4A27-63DE-4E60-95B6-FD63419CBE3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20" yWindow="20" windowWidth="19180" windowHeight="10060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Runtime" sheetId="1" r:id="rId1"/>
@@ -246,6 +246,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -254,12 +260,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -542,43 +542,43 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L75"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" customWidth="1"/>
-    <col min="2" max="12" width="12.6640625" customWidth="1"/>
+    <col min="1" max="1" width="12.54296875" customWidth="1"/>
+    <col min="2" max="12" width="12.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A3" s="15" t="s">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A3" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="13"/>
-      <c r="D3" s="12" t="s">
+      <c r="C3" s="15"/>
+      <c r="D3" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="14"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="12" t="s">
+      <c r="E3" s="16"/>
+      <c r="F3" s="15"/>
+      <c r="G3" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="H3" s="14"/>
-      <c r="I3" s="13"/>
-      <c r="J3" s="14" t="s">
+      <c r="H3" s="16"/>
+      <c r="I3" s="15"/>
+      <c r="J3" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="K3" s="14"/>
-      <c r="L3" s="14"/>
-    </row>
-    <row r="4" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="16"/>
+      <c r="K3" s="16"/>
+      <c r="L3" s="16"/>
+    </row>
+    <row r="4" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="13"/>
       <c r="B4" s="5" t="s">
         <v>7</v>
       </c>
@@ -613,7 +613,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" s="3">
         <v>10000000</v>
       </c>
@@ -644,7 +644,7 @@
         <v>1.3503039831807164</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" s="3">
         <v>11000000</v>
       </c>
@@ -675,7 +675,7 @@
         <v>1.4314321789308464</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7" s="3">
         <v>12000000</v>
       </c>
@@ -706,7 +706,7 @@
         <v>1.3990388485014549</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A8" s="3">
         <v>13000000</v>
       </c>
@@ -737,7 +737,7 @@
         <v>1.4162593677956241</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9" s="3">
         <v>14000000</v>
       </c>
@@ -768,7 +768,7 @@
         <v>1.4353413689728149</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A10" s="3">
         <v>15000000</v>
       </c>
@@ -799,7 +799,7 @@
         <v>1.4958510931601727</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A11" s="3">
         <v>16000000</v>
       </c>
@@ -830,7 +830,7 @@
         <v>1.4946658808534796</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A12" s="3">
         <v>17000000</v>
       </c>
@@ -861,7 +861,7 @@
         <v>1.5314277225416137</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A13" s="3">
         <v>18000000</v>
       </c>
@@ -892,7 +892,7 @@
         <v>1.7010684087007899</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A14" s="3">
         <v>19000000</v>
       </c>
@@ -923,7 +923,7 @@
         <v>1.8466274211032072</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A15" s="3">
         <v>20000000</v>
       </c>
@@ -954,7 +954,7 @@
         <v>1.9658831253344848</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A16" s="3">
         <v>21000000</v>
       </c>
@@ -985,7 +985,7 @@
         <v>1.6905367661533188</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" s="3">
         <v>22000000</v>
       </c>
@@ -1016,7 +1016,7 @@
         <v>1.4562076078036108</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" s="3">
         <v>23000000</v>
       </c>
@@ -1047,7 +1047,7 @@
         <v>1.4736406545695642</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" s="3">
         <v>24000000</v>
       </c>
@@ -1078,7 +1078,7 @@
         <v>1.5024524352787376</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20" s="3">
         <v>25000000</v>
       </c>
@@ -1109,7 +1109,7 @@
         <v>1.3807101680016927</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" s="3">
         <v>26000000</v>
       </c>
@@ -1140,7 +1140,7 @@
         <v>1.4815484367362499</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A22" s="3">
         <v>27000000</v>
       </c>
@@ -1171,7 +1171,7 @@
         <v>1.4320888444651907</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A23" s="3">
         <v>28000000</v>
       </c>
@@ -1202,7 +1202,7 @@
         <v>1.4896735870398701</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24" s="3">
         <v>29000000</v>
       </c>
@@ -1233,7 +1233,7 @@
         <v>1.4574478596011657</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A25" s="3">
         <v>30000000</v>
       </c>
@@ -1264,7 +1264,7 @@
         <v>1.471640083333507</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A26" s="3">
         <v>31000000</v>
       </c>
@@ -1295,7 +1295,7 @@
         <v>1.4480301190510056</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A27" s="3">
         <v>32000000</v>
       </c>
@@ -1326,7 +1326,7 @@
         <v>1.4799671594867332</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A28" s="3">
         <v>33000000</v>
       </c>
@@ -1357,7 +1357,7 @@
         <v>1.4870401475364317</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A29" s="3">
         <v>34000000</v>
       </c>
@@ -1388,7 +1388,7 @@
         <v>1.4523169715947184</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A30" s="3">
         <v>35000000</v>
       </c>
@@ -1419,7 +1419,7 @@
         <v>1.4342921380463396</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A31" s="3">
         <v>36000000</v>
       </c>
@@ -1450,7 +1450,7 @@
         <v>1.6968519767772656</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A32" s="3">
         <v>37000000</v>
       </c>
@@ -1481,7 +1481,7 @@
         <v>1.5276332531432211</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A33" s="3">
         <v>38000000</v>
       </c>
@@ -1512,7 +1512,7 @@
         <v>1.6903936314613837</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A34" s="3">
         <v>39000000</v>
       </c>
@@ -1543,7 +1543,7 @@
         <v>1.4135842256219358</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A35" s="3">
         <v>40000000</v>
       </c>
@@ -1574,38 +1574,38 @@
         <v>1.4963832739552605</v>
       </c>
     </row>
-    <row r="36" spans="1:12" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="37" spans="1:12" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:12" ht="40" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="37" spans="1:12" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A38" s="15" t="s">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A38" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="B38" s="12" t="s">
+      <c r="B38" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="C38" s="13"/>
-      <c r="D38" s="12" t="s">
+      <c r="C38" s="15"/>
+      <c r="D38" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="E38" s="14"/>
-      <c r="F38" s="13"/>
-      <c r="G38" s="12" t="s">
+      <c r="E38" s="16"/>
+      <c r="F38" s="15"/>
+      <c r="G38" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="H38" s="14"/>
-      <c r="I38" s="13"/>
-      <c r="J38" s="14" t="s">
+      <c r="H38" s="16"/>
+      <c r="I38" s="15"/>
+      <c r="J38" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="K38" s="14"/>
-      <c r="L38" s="14"/>
-    </row>
-    <row r="39" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="16"/>
+      <c r="K38" s="16"/>
+      <c r="L38" s="16"/>
+    </row>
+    <row r="39" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A39" s="13"/>
       <c r="B39" s="5" t="s">
         <v>7</v>
       </c>
@@ -1640,7 +1640,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A40" s="3">
         <v>10000000</v>
       </c>
@@ -1671,7 +1671,7 @@
         <v>1.2404784823894681</v>
       </c>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A41" s="3">
         <v>11000000</v>
       </c>
@@ -1702,7 +1702,7 @@
         <v>1.2744177730313988</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A42" s="3">
         <v>12000000</v>
       </c>
@@ -1733,7 +1733,7 @@
         <v>1.5768721682293738</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A43" s="3">
         <v>13000000</v>
       </c>
@@ -1764,7 +1764,7 @@
         <v>1.4027845914718184</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A44" s="3">
         <v>14000000</v>
       </c>
@@ -1795,7 +1795,7 @@
         <v>1.4486742368784218</v>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A45" s="3">
         <v>15000000</v>
       </c>
@@ -1826,7 +1826,7 @@
         <v>1.3330253848550908</v>
       </c>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A46" s="3">
         <v>16000000</v>
       </c>
@@ -1857,7 +1857,7 @@
         <v>1.5375576433617986</v>
       </c>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A47" s="3">
         <v>17000000</v>
       </c>
@@ -1888,7 +1888,7 @@
         <v>1.4187548742936833</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A48" s="3">
         <v>18000000</v>
       </c>
@@ -1919,7 +1919,7 @@
         <v>1.6579402664176821</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A49" s="3">
         <v>19000000</v>
       </c>
@@ -1950,7 +1950,7 @@
         <v>1.5085287104372207</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A50" s="3">
         <v>20000000</v>
       </c>
@@ -1981,7 +1981,7 @@
         <v>1.2742606830016989</v>
       </c>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A51" s="3">
         <v>21000000</v>
       </c>
@@ -2012,7 +2012,7 @@
         <v>1.4290755696529558</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A52" s="3">
         <v>22000000</v>
       </c>
@@ -2043,7 +2043,7 @@
         <v>1.5863120987088903</v>
       </c>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A53" s="3">
         <v>23000000</v>
       </c>
@@ -2074,7 +2074,7 @@
         <v>1.5483196236768955</v>
       </c>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A54" s="3">
         <v>24000000</v>
       </c>
@@ -2105,7 +2105,7 @@
         <v>1.3919663071986854</v>
       </c>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A55" s="3">
         <v>25000000</v>
       </c>
@@ -2136,7 +2136,7 @@
         <v>1.234497260335276</v>
       </c>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A56" s="3">
         <v>26000000</v>
       </c>
@@ -2167,7 +2167,7 @@
         <v>1.3742770690382931</v>
       </c>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A57" s="3">
         <v>27000000</v>
       </c>
@@ -2198,7 +2198,7 @@
         <v>2.02110536579108</v>
       </c>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A58" s="3">
         <v>28000000</v>
       </c>
@@ -2229,7 +2229,7 @@
         <v>1.52013082132216</v>
       </c>
     </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A59" s="3">
         <v>29000000</v>
       </c>
@@ -2260,7 +2260,7 @@
         <v>1.1606666840688113</v>
       </c>
     </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A60" s="3">
         <v>30000000</v>
       </c>
@@ -2291,7 +2291,7 @@
         <v>1.4818759670486334</v>
       </c>
     </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A61" s="3">
         <v>31000000</v>
       </c>
@@ -2322,7 +2322,7 @@
         <v>1.3800012599249023</v>
       </c>
     </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A62" s="3">
         <v>32000000</v>
       </c>
@@ -2353,7 +2353,7 @@
         <v>1.4434307699009739</v>
       </c>
     </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A63" s="3">
         <v>33000000</v>
       </c>
@@ -2384,7 +2384,7 @@
         <v>1.4095719197989531</v>
       </c>
     </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A64" s="3">
         <v>34000000</v>
       </c>
@@ -2415,7 +2415,7 @@
         <v>1.3299687295703455</v>
       </c>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A65" s="3">
         <v>35000000</v>
       </c>
@@ -2446,7 +2446,7 @@
         <v>1.4035055827925567</v>
       </c>
     </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A66" s="3">
         <v>36000000</v>
       </c>
@@ -2477,7 +2477,7 @@
         <v>1.3064700586106652</v>
       </c>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A67" s="3">
         <v>37000000</v>
       </c>
@@ -2508,7 +2508,7 @@
         <v>1.4599944828606854</v>
       </c>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A68" s="3">
         <v>38000000</v>
       </c>
@@ -2539,7 +2539,7 @@
         <v>1.6088829324692671</v>
       </c>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A69" s="3">
         <v>39000000</v>
       </c>
@@ -2570,7 +2570,7 @@
         <v>1.4417550579449547</v>
       </c>
     </row>
-    <row r="70" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A70" s="3">
         <v>40000000</v>
       </c>
@@ -2601,23 +2601,23 @@
         <v>1.8097493762345969</v>
       </c>
     </row>
-    <row r="75" spans="1:9" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:9" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A75" s="7" t="s">
         <v>11</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="D3:F3"/>
+    <mergeCell ref="G3:I3"/>
+    <mergeCell ref="J3:L3"/>
+    <mergeCell ref="A3:A4"/>
     <mergeCell ref="A38:A39"/>
     <mergeCell ref="B38:C38"/>
     <mergeCell ref="D38:F38"/>
     <mergeCell ref="G38:I38"/>
     <mergeCell ref="J38:L38"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="D3:F3"/>
-    <mergeCell ref="G3:I3"/>
-    <mergeCell ref="J3:L3"/>
-    <mergeCell ref="A3:A4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>